<commit_message>
Recuperar avisos del BORA de 4 días que quedaron vacíos (31/7, 31/8, 11/9, 6/10)
El robot no pudo leer el BORA esos días. Se bajaron las ediciones de esas fechas
y se conservaron los datos de Comprar y TGN que ya se habían guardado ese día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VmfpwzVWvRWhRHG7VzpiEN
</commit_message>
<xml_diff>
--- a/data/2026-07/flujo_licitaciones_2026-07-31.xlsx
+++ b/data/2026-07/flujo_licitaciones_2026-07-31.xlsx
@@ -7,7 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⏳ Licitaciones Abiertas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="✅ Adjudicados con CUIT" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔗 Flujo Cruzado" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💰 Cobraron en TGN" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⏳ Licitaciones Abiertas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,6 +416,965 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fecha_extraccion</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>fecha_publicacion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>organismo_contratante</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>tipo_proceso</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>aviso_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>proveedor_adjudicado</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>cuit_proveedor</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>monto_adjudicado</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>texto_muestra</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO - DIRECCIÓN REGIONAL ADUANERA CUYO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Licitación Pública 04/26</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2415305</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/tercera/2415305/20260731</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>CONFECCIONES JOSÉ CONTARTESE Y CIA S.R.L</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>30-52141731-1</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>$22.374.000,00</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/pdf/linkQR/b3JqdlBNaXVoVVJSbkVWUVVZR3c4dz09
+AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO -
+DIRECCIÓN REGIONAL ADUANERA CUYO
+Licitación Pública 04/26
+Expediente  Nº:  EX-2026-02324707-  -ARCA-SECFDVAFCU#SDGOAI  Objeto  de  la  contratación:
+Adquisición  de  indumenta</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>BORA Adjudicaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO - DIRECCIÓN REGIONAL ADUANERA HIDROVÍA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Licitación Pública 22/2026</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2415306</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/tercera/2415306/20260731</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>MERCOSUR SEGURIDAD S.R.L</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>30-71070541-7</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>$170.820.000,00</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/pdf/linkQR/eVJmRkpwajRFUVJSbkVWUVVZR3c4dz09
+AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO -
+DIRECCIÓN REGIONAL ADUANERA HIDROVÍA
+Licitación Pública 22/2026
+Ejercicio:  2026  Expediente  Nº:  EX-2026-01254739--ARCA-SECFDVAFHI#SDGOAI  Objeto  de  la
+contratación: “SERV</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>BORA Adjudicaciones</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>organismo_contratante</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>tipo_proceso_bora</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>link_bora</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>proveedor_adjudicado</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>cuit_proveedor</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>monto_adjudicado_bora</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>en_comprar</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>procesos_comprar</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>unidad_comprar</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>nro_proceso_comprar</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>cobro_en_tgn</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>beneficiario_tgn</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>monto_cobrado_tgn</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>metodo_cruce_tgn</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>etapa</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>alerta</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>indicadores_riesgo</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>score_riesgo_licit</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>indice_riesgo_licit</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>nivel_riesgo_licit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO - DIRECCIÓN REGIONAL ADUANERA CUYO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Licitación Pública 04/26</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/tercera/2415305/20260731</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CONFECCIONES JOSÉ CONTARTESE Y CIA S.R.L</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>30-52141731-1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>$22.374.000,00</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>❌ NO</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>✅ SÍ</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Administración de Parques Nacionales</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>43.90238429</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>organismo</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>💰 ADJUDICADO + ORGANISMO CON PAGOS TGN</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>🔶 BORA + TGN (por organismo)</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>✅ Sin alertas</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO - DIRECCIÓN REGIONAL ADUANERA HIDROVÍA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Licitación Pública 22/2026</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/tercera/2415306/20260731</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MERCOSUR SEGURIDAD S.R.L</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>30-71070541-7</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>$170.820.000,00</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>❌ NO</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>✅ SÍ</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Administración de Parques Nacionales</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>43.90238429</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>organismo</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>💰 ADJUDICADO + ORGANISMO CON PAGOS TGN</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>🔶 BORA + TGN (por organismo)</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>✅ Sin alertas</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ADMINISTRACIÓN NACIONAL DE LA SEGURIDAD SOCIAL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Licitación Pública PROCESO COMPR.AR 63-0082-LPU25</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/tercera/2415307/20260731</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>❌ NO</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>✅ SÍ</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Administración Nacional de Aviación Civil</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>3366.71186018</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>organismo</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>⚠️ SIN CUIT EXTRAÍDO</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>🔶 BORA + TGN (por organismo)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>✅ Sin alertas</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>organismo_contratante</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>tipo_proceso_bora</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>link_bora</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>proveedor_adjudicado</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>cuit_proveedor</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>monto_adjudicado_bora</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>en_comprar</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>procesos_comprar</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>unidad_comprar</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>nro_proceso_comprar</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>cobro_en_tgn</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>beneficiario_tgn</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>monto_cobrado_tgn</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>metodo_cruce_tgn</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>etapa</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>alerta</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>indicadores_riesgo</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>score_riesgo_licit</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>indice_riesgo_licit</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>nivel_riesgo_licit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO - DIRECCIÓN REGIONAL ADUANERA CUYO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Licitación Pública 04/26</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/tercera/2415305/20260731</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CONFECCIONES JOSÉ CONTARTESE Y CIA S.R.L</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>30-52141731-1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>$22.374.000,00</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>❌ NO</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>✅ SÍ</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Administración de Parques Nacionales</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>43.90238429</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>organismo</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>💰 ADJUDICADO + ORGANISMO CON PAGOS TGN</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>🔶 BORA + TGN (por organismo)</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>✅ Sin alertas</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO - DIRECCIÓN REGIONAL ADUANERA HIDROVÍA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Licitación Pública 22/2026</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/tercera/2415306/20260731</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MERCOSUR SEGURIDAD S.R.L</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>30-71070541-7</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>$170.820.000,00</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>❌ NO</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>✅ SÍ</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Administración de Parques Nacionales</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>43.90238429</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>organismo</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>💰 ADJUDICADO + ORGANISMO CON PAGOS TGN</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>🔶 BORA + TGN (por organismo)</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>✅ Sin alertas</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ADMINISTRACIÓN NACIONAL DE LA SEGURIDAD SOCIAL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Licitación Pública PROCESO COMPR.AR 63-0082-LPU25</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/tercera/2415307/20260731</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>❌ NO</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>✅ SÍ</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Administración Nacional de Aviación Civil</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>3366.71186018</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>organismo</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>⚠️ SIN CUIT EXTRAÍDO</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>🔶 BORA + TGN (por organismo)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>✅ Sin alertas</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>